<commit_message>
Plantilla de novedades: tipos NOTIFICACION y MERMA
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_011eGKqn2gUS8cs5eYR1TxLK
</commit_message>
<xml_diff>
--- a/public/plantillas/analisis-diferencia-novedades.xlsx
+++ b/public/plantillas/analisis-diferencia-novedades.xlsx
@@ -11277,18 +11277,58 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>NOTIFICACION</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>CONTEO</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente notificación de envase: existe, suma al conteo.</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>MERMA</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>CONTEO</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Merma de envase: suma al conteo.</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>

</xml_diff>

<commit_message>
Análisis de diferencia: la DEPA de cada línea se puede subir en la plantilla cuando no hay corte inicial
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_011eGKqn2gUS8cs5eYR1TxLK
</commit_message>
<xml_diff>
--- a/public/plantillas/analisis-diferencia-novedades.xlsx
+++ b/public/plantillas/analisis-diferencia-novedades.xlsx
@@ -581,7 +581,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Llena solo lo amarillo: el tipo, el código y la cantidad (en estibas, cajas o unidades: la que tengas). N° de entrega solo en PEND NOVEDADES CD. La ZEXI de las 6 va aquí también (tipo ZEXI 6 AM, en UNIDADES SUELTAS). Lo gris sale solo; VALIDACIÓN debe decir OK.</t>
+          <t>Llena solo lo amarillo: el tipo, el código y la cantidad (en estibas, cajas o unidades: la que tengas). N° de entrega solo en PEND NOVEDADES CD. La ZEXI de las 6 va aquí también (tipo ZEXI 6 AM, en UNIDADES SUELTAS). La DEPA de cada línea (tipo DEPA L1, DEPA L2, DEPA L4, DEPA L6, en UNIDADES SUELTAS o estibas/cajas) también va aquí cuando no hay corte inicial ese día. Lo gris sale solo; VALIDACIÓN debe decir OK.</t>
         </is>
       </c>
     </row>
@@ -10281,7 +10281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10508,7 +10508,33 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>DEPA L1</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n">
+        <v>3500005</v>
+      </c>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n">
+        <v>330714</v>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>330.714 u</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>3500231 · 8.703</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Las cajas plásticas NO se escriben aparte: salen solas del envase (2052/38, 39780/30… como en tu Excel).</t>
         </is>
@@ -11331,32 +11357,112 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>DEPA L1</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>CONTEO</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Depaletizadora de la línea L1: lo que marca la depa. Solo si NO hay corte inicial ese día (si lo hay, la app usa el corte). La caja plástica sale sola del envase.</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>DEPA L2</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>CONTEO</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>Depaletizadora de la línea L2: lo que marca la depa. Solo si NO hay corte inicial ese día (si lo hay, la app usa el corte). La caja plástica sale sola del envase.</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>DEPA L4</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>CONTEO</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>Depaletizadora de la línea L4: lo que marca la depa. Solo si NO hay corte inicial ese día (si lo hay, la app usa el corte). La caja plástica sale sola del envase.</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>DEPA L6</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>CONTEO</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Depaletizadora de la línea L6: lo que marca la depa. Solo si NO hay corte inicial ese día (si lo hay, la app usa el corte). La caja plástica sale sola del envase.</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>

</xml_diff>